<commit_message>
add features and interactive sheet
</commit_message>
<xml_diff>
--- a/facial-attendance/data/students.xlsx
+++ b/facial-attendance/data/students.xlsx
@@ -434,12 +434,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C2"/>
+  <dimension ref="A1:D2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
     <col width="24" customWidth="1" min="2" max="2"/>
     <col width="24" customWidth="1" min="3" max="3"/>
+    <col width="24" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -458,11 +459,16 @@
           <t>photo_path</t>
         </is>
       </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>id_card_path</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>101</t>
+          <t>3147</t>
         </is>
       </c>
       <c r="B2" s="3" t="inlineStr">
@@ -472,7 +478,12 @@
       </c>
       <c r="C2" s="3" t="inlineStr">
         <is>
-          <t>photos/101.jpg</t>
+          <t>photos/3147.jpg</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="inlineStr">
+        <is>
+          <t>id_cards/3147.jpg</t>
         </is>
       </c>
     </row>

</xml_diff>